<commit_message>
Test Data Updated by Mahesh
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2521763_cognizant_com/Documents/Desktop/onepointtest/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521834\Downloads\onepoint_testing\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="8_{34392B7F-6071-4B3B-92E7-75E38F1EF913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F423AA9-0910-4200-9B5B-A6003BAF6BF6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89AED0C2-3C80-4EF0-AFAE-E103F79BB16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{9E738272-3848-4331-9E3A-383B4E062269}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{9E738272-3848-4331-9E3A-383B4E062269}"/>
   </bookViews>
   <sheets>
     <sheet name="Response_Submission" sheetId="1" r:id="rId1"/>
+    <sheet name="Template_Form_Creation" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="121">
   <si>
     <t>TC ID</t>
   </si>
@@ -199,12 +200,222 @@
   <si>
     <t>System follows the application's configured duplicate-submission rule: duplicate is blocked or handled according to the implemented behavior.</t>
   </si>
+  <si>
+    <t>Page / URL</t>
+  </si>
+  <si>
+    <t>Template Selected</t>
+  </si>
+  <si>
+    <t>Form Title</t>
+  </si>
+  <si>
+    <t>Form Description</t>
+  </si>
+  <si>
+    <t>Question Action</t>
+  </si>
+  <si>
+    <t>Question Label</t>
+  </si>
+  <si>
+    <t>Field Type</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>Distribution Type</t>
+  </si>
+  <si>
+    <t>Response Limit Cap</t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>Expiry Date</t>
+  </si>
+  <si>
+    <t>Save Action</t>
+  </si>
+  <si>
+    <t>TC03-01</t>
+  </si>
+  <si>
+    <t>https://one-point-jet.vercel.app/templates</t>
+  </si>
+  <si>
+    <t>Templates page opens and all 7 templates are displayed.</t>
+  </si>
+  <si>
+    <t>TC03-02</t>
+  </si>
+  <si>
+    <t>Employee Feedback Form</t>
+  </si>
+  <si>
+    <t>Click Use Template</t>
+  </si>
+  <si>
+    <t>Selected template opens successfully in form builder.</t>
+  </si>
+  <si>
+    <t>TC03-03</t>
+  </si>
+  <si>
+    <t>Employee Pulse &amp; Culture Feedback</t>
+  </si>
+  <si>
+    <t>Anonymous survey to evaluate employee workplace morale and culture.</t>
+  </si>
+  <si>
+    <t>Review loaded content</t>
+  </si>
+  <si>
+    <t>Q1,Q2,Q3</t>
+  </si>
+  <si>
+    <t>Star/NPS; Checkbox; Textarea</t>
+  </si>
+  <si>
+    <t>Q1 Yes; Q2 No; Q3 Yes</t>
+  </si>
+  <si>
+    <t>Template content loads correctly.</t>
+  </si>
+  <si>
+    <t>TC03-04</t>
+  </si>
+  <si>
+    <t>Edit Q1 label</t>
+  </si>
+  <si>
+    <t>Overall Job Satisfaction Level</t>
+  </si>
+  <si>
+    <t>Star / NPS Rating</t>
+  </si>
+  <si>
+    <t>Save as Draft</t>
+  </si>
+  <si>
+    <t>Modified Q1 label is saved and retained.</t>
+  </si>
+  <si>
+    <t>TC03-05</t>
+  </si>
+  <si>
+    <t>Add Question to Section 1</t>
+  </si>
+  <si>
+    <t>Phone Number</t>
+  </si>
+  <si>
+    <t>Short Text</t>
+  </si>
+  <si>
+    <t>New question appears after save.</t>
+  </si>
+  <si>
+    <t>TC03-06</t>
+  </si>
+  <si>
+    <t>Delete Q3</t>
+  </si>
+  <si>
+    <t>Multi-Line Textarea</t>
+  </si>
+  <si>
+    <t>Q3 is removed after save/reopen.</t>
+  </si>
+  <si>
+    <t>TC03-07</t>
+  </si>
+  <si>
+    <t>Q4 Employee Culture Survey</t>
+  </si>
+  <si>
+    <t>Change form title</t>
+  </si>
+  <si>
+    <t>New form title retained.</t>
+  </si>
+  <si>
+    <t>TC03-07a</t>
+  </si>
+  <si>
+    <t>(empty)</t>
+  </si>
+  <si>
+    <t>Clear form title</t>
+  </si>
+  <si>
+    <t>Save blocked with validation.</t>
+  </si>
+  <si>
+    <t>Invalid</t>
+  </si>
+  <si>
+    <t>TC03-08</t>
+  </si>
+  <si>
+    <t>Edit Q1 label + Add Phone Number</t>
+  </si>
+  <si>
+    <t>Overall Job Satisfaction Level; Phone Number</t>
+  </si>
+  <si>
+    <t>Star/NPS; Short Text</t>
+  </si>
+  <si>
+    <t>Yes; No</t>
+  </si>
+  <si>
+    <t>Internal Employees Only</t>
+  </si>
+  <si>
+    <t>Customized form saved with DRAFT status.</t>
+  </si>
+  <si>
+    <t>TC03-09</t>
+  </si>
+  <si>
+    <t>https://one-point-jet.vercel.app/forms</t>
+  </si>
+  <si>
+    <t>Open saved form</t>
+  </si>
+  <si>
+    <t>All customizations retained.</t>
+  </si>
+  <si>
+    <t>TC03-10 First Form</t>
+  </si>
+  <si>
+    <t>TC03_10_FORM_A</t>
+  </si>
+  <si>
+    <t>TC03_10_FORM_A_Q1</t>
+  </si>
+  <si>
+    <t>First form created and saved.</t>
+  </si>
+  <si>
+    <t>TC03-10 Second Form</t>
+  </si>
+  <si>
+    <t>Click Use Template again</t>
+  </si>
+  <si>
+    <t>Second form starts from original template.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,7 +436,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -244,8 +455,14 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -288,11 +505,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -311,6 +543,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -647,17 +888,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6FC487B-C59D-44B2-9724-B633962AB9D6}">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
-    <col min="3" max="3" width="33.5703125" customWidth="1"/>
-    <col min="4" max="4" width="38.140625" customWidth="1"/>
-    <col min="5" max="5" width="42.85546875" customWidth="1"/>
-    <col min="6" max="6" width="27.42578125" customWidth="1"/>
+    <col min="2" max="2" width="31.26953125" customWidth="1"/>
+    <col min="3" max="3" width="33.54296875" customWidth="1"/>
+    <col min="4" max="4" width="38.1796875" customWidth="1"/>
+    <col min="5" max="5" width="42.81640625" customWidth="1"/>
+    <col min="6" max="6" width="27.453125" customWidth="1"/>
     <col min="7" max="7" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="29.1">
+    <row r="1" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -683,7 +924,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="43.5">
+    <row r="2" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -709,7 +950,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="106.5">
+    <row r="3" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
@@ -735,7 +976,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="43.5">
+    <row r="4" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
@@ -761,7 +1002,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="43.5">
+    <row r="5" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
@@ -785,7 +1026,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="43.5">
+    <row r="6" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -805,7 +1046,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="43.5">
+    <row r="7" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>29</v>
       </c>
@@ -831,7 +1072,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="43.5">
+    <row r="8" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>32</v>
       </c>
@@ -857,7 +1098,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="43.5">
+    <row r="9" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>37</v>
       </c>
@@ -883,7 +1124,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="43.5">
+    <row r="10" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
@@ -909,7 +1150,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="57.95">
+    <row r="11" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>45</v>
       </c>
@@ -935,7 +1176,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="57.95">
+    <row r="12" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>49</v>
       </c>
@@ -965,4 +1206,590 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToWidth="0" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9001167C-3461-4628-8CBA-85AA4DD8F878}">
+  <dimension ref="A1:P13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.90625" customWidth="1"/>
+    <col min="2" max="2" width="36.54296875" customWidth="1"/>
+    <col min="3" max="3" width="35.08984375" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="5" max="5" width="22.54296875" customWidth="1"/>
+    <col min="6" max="6" width="21.1796875" customWidth="1"/>
+    <col min="7" max="7" width="20.54296875" customWidth="1"/>
+    <col min="8" max="8" width="23.26953125" customWidth="1"/>
+    <col min="9" max="9" width="15.453125" customWidth="1"/>
+    <col min="10" max="10" width="16.453125" customWidth="1"/>
+    <col min="11" max="11" width="19.26953125" customWidth="1"/>
+    <col min="12" max="12" width="15.26953125" customWidth="1"/>
+    <col min="13" max="13" width="15.90625" customWidth="1"/>
+    <col min="14" max="14" width="13.6328125" customWidth="1"/>
+    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="16" max="16" width="15.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="116" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="P2" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="P3" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="145" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="P4" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="P6" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="116" x14ac:dyDescent="0.35">
+      <c r="A7" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="P7" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="P8" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="O9" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="P9" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="87" x14ac:dyDescent="0.35">
+      <c r="A10" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="K10" s="8">
+        <v>250</v>
+      </c>
+      <c r="L10" s="9">
+        <v>46305.375</v>
+      </c>
+      <c r="M10" s="9">
+        <v>46336.75</v>
+      </c>
+      <c r="N10" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="P10" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="87" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="K11" s="8">
+        <v>250</v>
+      </c>
+      <c r="L11" s="9">
+        <v>46305.375</v>
+      </c>
+      <c r="M11" s="9">
+        <v>46336.75</v>
+      </c>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="P11" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="O12" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="P12" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="P13" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Test Data updated by Rohan
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521834\Downloads\onepoint_testing\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2521758_cognizant_com/Documents/Desktop/onepoint_testing/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89AED0C2-3C80-4EF0-AFAE-E103F79BB16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{89AED0C2-3C80-4EF0-AFAE-E103F79BB16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16A0F4A8-C5C0-497C-84A2-1852B8839E0C}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{9E738272-3848-4331-9E3A-383B4E062269}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{9E738272-3848-4331-9E3A-383B4E062269}"/>
   </bookViews>
   <sheets>
     <sheet name="Response_Submission" sheetId="1" r:id="rId1"/>
     <sheet name="Template_Form_Creation" sheetId="2" r:id="rId2"/>
+    <sheet name="Response_Analysis" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="187">
   <si>
     <t>TC ID</t>
   </si>
@@ -409,6 +410,204 @@
   </si>
   <si>
     <t>Second form starts from original template.</t>
+  </si>
+  <si>
+    <t>Navigation / Action</t>
+  </si>
+  <si>
+    <t>Submission / Test Data</t>
+  </si>
+  <si>
+    <t>Value to Verify</t>
+  </si>
+  <si>
+    <t>TC05-01</t>
+  </si>
+  <si>
+    <t>Login as Admin (EMP001) → Dashboard → More actions → Responses</t>
+  </si>
+  <si>
+    <t>Heading: Form Analytics: Employee Pulse &amp; Culture Feedback</t>
+  </si>
+  <si>
+    <t>Response Analysis page opens successfully and shows the form title, metric cards, question-wise analysis and submissions table.</t>
+  </si>
+  <si>
+    <t>TC05-02</t>
+  </si>
+  <si>
+    <t>Read Total Submissions card and heading</t>
+  </si>
+  <si>
+    <t>Valid submissions from TC04</t>
+  </si>
+  <si>
+    <t>Total Submissions equals valid submissions count</t>
+  </si>
+  <si>
+    <t>Total Submissions, heading count and table rows match submitted responses.</t>
+  </si>
+  <si>
+    <t>TC05-03</t>
+  </si>
+  <si>
+    <t>Submissions table → Inspect Answers</t>
+  </si>
+  <si>
+    <t>Any one submission</t>
+  </si>
+  <si>
+    <t>Popup title: Submission Detail</t>
+  </si>
+  <si>
+    <t>Popup shows respondent, submission date/time and all answers.</t>
+  </si>
+  <si>
+    <t>TC05-04</t>
+  </si>
+  <si>
+    <t>Inspect Answers on TC04-09 submission</t>
+  </si>
+  <si>
+    <t>Submitted values match TC04-09 data</t>
+  </si>
+  <si>
+    <t>Each answer exactly matches submitted values.</t>
+  </si>
+  <si>
+    <t>TC05-05</t>
+  </si>
+  <si>
+    <t>Inspect answers on each row</t>
+  </si>
+  <si>
+    <t>TC04-03, TC04-07, TC04-08, TC04-09, TC04-10</t>
+  </si>
+  <si>
+    <t>Improvement texts match submitted records</t>
+  </si>
+  <si>
+    <t>Every response listed with correct answers.</t>
+  </si>
+  <si>
+    <t>TC05-06</t>
+  </si>
+  <si>
+    <t>Review metric cards and analysis section</t>
+  </si>
+  <si>
+    <t>All TC04 valid submissions</t>
+  </si>
+  <si>
+    <t>Average rating = 3.8/5.0</t>
+  </si>
+  <si>
+    <t>Metrics and counts match data.</t>
+  </si>
+  <si>
+    <t>TC05-07</t>
+  </si>
+  <si>
+    <t>Submit new response and refresh</t>
+  </si>
+  <si>
+    <t>Rating 4; Career Growth; NEW_TC05_07</t>
+  </si>
+  <si>
+    <t>Count increases by 1</t>
+  </si>
+  <si>
+    <t>New submission appears correctly.</t>
+  </si>
+  <si>
+    <t>TC05-08</t>
+  </si>
+  <si>
+    <t>Link of empty form</t>
+  </si>
+  <si>
+    <t>Open Responses on empty form</t>
+  </si>
+  <si>
+    <t>Form with 0 submissions</t>
+  </si>
+  <si>
+    <t>Total Submissions = 0</t>
+  </si>
+  <si>
+    <t>Shows empty-state message without errors.</t>
+  </si>
+  <si>
+    <t>TC05-09</t>
+  </si>
+  <si>
+    <t>Click Export CSV</t>
+  </si>
+  <si>
+    <t>All submissions</t>
+  </si>
+  <si>
+    <t>Downloaded CSV count = Total Submissions</t>
+  </si>
+  <si>
+    <t>CSV downloads with all responses.</t>
+  </si>
+  <si>
+    <t>TC05-10</t>
+  </si>
+  <si>
+    <t>Click Export Excel</t>
+  </si>
+  <si>
+    <t>Downloaded XLSX count = Total Submissions</t>
+  </si>
+  <si>
+    <t>Excel downloads and opens correctly.</t>
+  </si>
+  <si>
+    <t>TC05-11</t>
+  </si>
+  <si>
+    <t>Click Export PDF</t>
+  </si>
+  <si>
+    <t>PDF shows form title and responses</t>
+  </si>
+  <si>
+    <t>PDF downloads and opens correctly.</t>
+  </si>
+  <si>
+    <t>TC05-12</t>
+  </si>
+  <si>
+    <t>Logout and open analytics URL directly</t>
+  </si>
+  <si>
+    <t>Not logged in</t>
+  </si>
+  <si>
+    <t>Redirect to login page</t>
+  </si>
+  <si>
+    <t>Analysis page not shown; redirected to Sign In.</t>
+  </si>
+  <si>
+    <t>TC05-13</t>
+  </si>
+  <si>
+    <t>https://one-point-jet.vercel.app/analytics/99999</t>
+  </si>
+  <si>
+    <t>Open non-existent form ID</t>
+  </si>
+  <si>
+    <t>Non-existent form ID</t>
+  </si>
+  <si>
+    <t>No response data shown</t>
+  </si>
+  <si>
+    <t>Shows error/not-found safely.</t>
   </si>
 </sst>
 </file>
@@ -436,7 +635,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -461,8 +660,13 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -520,11 +724,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -552,6 +771,12 @@
     </xf>
     <xf numFmtId="22" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1431,7 +1656,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>79</v>
       </c>
@@ -1471,7 +1696,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>85</v>
       </c>
@@ -1511,7 +1736,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="116" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>90</v>
       </c>
@@ -1551,7 +1776,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
         <v>94</v>
       </c>
@@ -1585,7 +1810,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>98</v>
       </c>
@@ -1619,7 +1844,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="87" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>103</v>
       </c>
@@ -1667,7 +1892,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="87" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>110</v>
       </c>
@@ -1713,7 +1938,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
         <v>114</v>
       </c>
@@ -1753,7 +1978,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
         <v>118</v>
       </c>
@@ -1792,4 +2017,345 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DFDEC2C-3E65-4E52-926E-AF0CF56FD70A}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.453125" customWidth="1"/>
+    <col min="2" max="2" width="59.90625" customWidth="1"/>
+    <col min="3" max="3" width="37.54296875" customWidth="1"/>
+    <col min="4" max="4" width="29.26953125" customWidth="1"/>
+    <col min="5" max="5" width="43.1796875" customWidth="1"/>
+    <col min="6" max="6" width="33.453125" customWidth="1"/>
+    <col min="7" max="7" width="11.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A5" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A6" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A7" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A8" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+      <c r="A9" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A10" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A11" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A12" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+      <c r="A13" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+      <c r="A14" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Test Data updated by Manogna
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2521758_cognizant_com/Documents/Desktop/onepoint_testing/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2521761_cognizant_com/Documents/Desktop/onepoint_testing/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{89AED0C2-3C80-4EF0-AFAE-E103F79BB16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16A0F4A8-C5C0-497C-84A2-1852B8839E0C}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{89AED0C2-3C80-4EF0-AFAE-E103F79BB16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{233B09AC-FB07-4C9C-963D-15419D0DE677}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{9E738272-3848-4331-9E3A-383B4E062269}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="3" xr2:uid="{9E738272-3848-4331-9E3A-383B4E062269}"/>
   </bookViews>
   <sheets>
     <sheet name="Response_Submission" sheetId="1" r:id="rId1"/>
     <sheet name="Template_Form_Creation" sheetId="2" r:id="rId2"/>
     <sheet name="Response_Analysis" sheetId="3" r:id="rId3"/>
+    <sheet name="Login_Details" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="212">
   <si>
     <t>TC ID</t>
   </si>
@@ -608,6 +609,81 @@
   </si>
   <si>
     <t>Shows error/not-found safely.</t>
+  </si>
+  <si>
+    <t>Test ID</t>
+  </si>
+  <si>
+    <t>Test Case Scenario</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>TC01</t>
+  </si>
+  <si>
+    <t>Login using valid employee credentials</t>
+  </si>
+  <si>
+    <t>EMP001</t>
+  </si>
+  <si>
+    <t>Password@123</t>
+  </si>
+  <si>
+    <t>Dashboard opens successfully.</t>
+  </si>
+  <si>
+    <t>TC02</t>
+  </si>
+  <si>
+    <t>Login using valid HR credentials</t>
+  </si>
+  <si>
+    <t>EMP002</t>
+  </si>
+  <si>
+    <t>TC03</t>
+  </si>
+  <si>
+    <t>Login with an incorrect password</t>
+  </si>
+  <si>
+    <t>wrong123</t>
+  </si>
+  <si>
+    <t>Login error message is displayed.</t>
+  </si>
+  <si>
+    <t>TC04</t>
+  </si>
+  <si>
+    <t>Login without entering username</t>
+  </si>
+  <si>
+    <t>Employee ID/email required validation is displayed.</t>
+  </si>
+  <si>
+    <t>TC05</t>
+  </si>
+  <si>
+    <t>Login without entering password</t>
+  </si>
+  <si>
+    <t>Password required validation is displayed.</t>
+  </si>
+  <si>
+    <t>TC06</t>
+  </si>
+  <si>
+    <t>Login with both username and password blank</t>
+  </si>
+  <si>
+    <t>Required-field validation is displayed and login is blocked.</t>
   </si>
 </sst>
 </file>
@@ -635,7 +711,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -665,8 +741,14 @@
         <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -739,11 +821,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -778,6 +875,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1606,7 +1705,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="145" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>71</v>
       </c>
@@ -2056,7 +2155,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="246.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
         <v>124</v>
       </c>
@@ -2079,7 +2178,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>128</v>
       </c>
@@ -2102,7 +2201,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
         <v>133</v>
       </c>
@@ -2125,7 +2224,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
         <v>138</v>
       </c>
@@ -2148,7 +2247,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>142</v>
       </c>
@@ -2171,7 +2270,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>147</v>
       </c>
@@ -2194,7 +2293,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
         <v>152</v>
       </c>
@@ -2217,7 +2316,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>157</v>
       </c>
@@ -2240,7 +2339,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
         <v>163</v>
       </c>
@@ -2263,7 +2362,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
         <v>168</v>
       </c>
@@ -2286,7 +2385,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
         <v>172</v>
       </c>
@@ -2309,7 +2408,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
         <v>176</v>
       </c>
@@ -2332,7 +2431,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
         <v>181</v>
       </c>
@@ -2353,6 +2452,156 @@
       </c>
       <c r="G14" s="11" t="s">
         <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{148981C6-6D91-479D-8C79-934D1547ACB0}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.1796875" customWidth="1"/>
+    <col min="2" max="2" width="38.1796875" customWidth="1"/>
+    <col min="3" max="3" width="16.36328125" customWidth="1"/>
+    <col min="4" max="4" width="18.54296875" customWidth="1"/>
+    <col min="5" max="5" width="47.36328125" customWidth="1"/>
+    <col min="6" max="6" width="13.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Test data update by Divya
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2521761_cognizant_com/Documents/Desktop/onepoint_testing/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521742\Desktop\onepoint_testing\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{89AED0C2-3C80-4EF0-AFAE-E103F79BB16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{233B09AC-FB07-4C9C-963D-15419D0DE677}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8533B1-8780-41BD-8A5B-3961A2BC0375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="3" xr2:uid="{9E738272-3848-4331-9E3A-383B4E062269}"/>
+    <workbookView xWindow="1760" yWindow="1800" windowWidth="15640" windowHeight="9370" firstSheet="2" activeTab="4" xr2:uid="{9E738272-3848-4331-9E3A-383B4E062269}"/>
   </bookViews>
   <sheets>
     <sheet name="Response_Submission" sheetId="1" r:id="rId1"/>
     <sheet name="Template_Form_Creation" sheetId="2" r:id="rId2"/>
     <sheet name="Response_Analysis" sheetId="3" r:id="rId3"/>
     <sheet name="Login_Details" sheetId="4" r:id="rId4"/>
+    <sheet name="BlankForm_creation" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="295">
   <si>
     <t>TC ID</t>
   </si>
@@ -684,6 +685,255 @@
   </si>
   <si>
     <t>Required-field validation is displayed and login is blocked.</t>
+  </si>
+  <si>
+    <t>TC_ID</t>
+  </si>
+  <si>
+    <t>Form_Title</t>
+  </si>
+  <si>
+    <t>Anonymous Submission</t>
+  </si>
+  <si>
+    <t>Response Limit</t>
+  </si>
+  <si>
+    <t>Section Name</t>
+  </si>
+  <si>
+    <t>Section Description</t>
+  </si>
+  <si>
+    <t>TC_001</t>
+  </si>
+  <si>
+    <t>Employee satisfaction survey</t>
+  </si>
+  <si>
+    <t>Public Link &amp; QR Code</t>
+  </si>
+  <si>
+    <t>Employee Details</t>
+  </si>
+  <si>
+    <t>Basic employee information</t>
+  </si>
+  <si>
+    <t>Full Name</t>
+  </si>
+  <si>
+    <t>Form should be published successfully</t>
+  </si>
+  <si>
+    <t>TC_002</t>
+  </si>
+  <si>
+    <t>Customer Survey</t>
+  </si>
+  <si>
+    <t>Survey for product review</t>
+  </si>
+  <si>
+    <t>Customer Details</t>
+  </si>
+  <si>
+    <t>Customer information</t>
+  </si>
+  <si>
+    <t>Email Address</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>Registration Form</t>
+  </si>
+  <si>
+    <t>Internal Users</t>
+  </si>
+  <si>
+    <t>Participant Info</t>
+  </si>
+  <si>
+    <t>Collect participant details</t>
+  </si>
+  <si>
+    <t>Mobile Number</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>Description available</t>
+  </si>
+  <si>
+    <t>Main Section</t>
+  </si>
+  <si>
+    <t>Section desc</t>
+  </si>
+  <si>
+    <t>Validation message should appear for Form Title</t>
+  </si>
+  <si>
+    <t>TC_006</t>
+  </si>
+  <si>
+    <t>@#$%^&amp;*</t>
+  </si>
+  <si>
+    <t>Invalid title test</t>
+  </si>
+  <si>
+    <t>Error should be shown for invalid Form Title</t>
+  </si>
+  <si>
+    <t>TC_007</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Single character title</t>
+  </si>
+  <si>
+    <t>Validation should appear if minimum length exists</t>
+  </si>
+  <si>
+    <t>TC_008</t>
+  </si>
+  <si>
+    <t>Very Long Form Title Exceeding Expected Application Limits To Verify Boundary Conditions And Length Validation</t>
+  </si>
+  <si>
+    <t>Desc</t>
+  </si>
+  <si>
+    <t>Validation should appear for title length</t>
+  </si>
+  <si>
+    <t>TC_009</t>
+  </si>
+  <si>
+    <t>Feedback Form</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Feedback Section</t>
+  </si>
+  <si>
+    <t>Feedback Details</t>
+  </si>
+  <si>
+    <t>Rating</t>
+  </si>
+  <si>
+    <t>Response Limit should reject negative values</t>
+  </si>
+  <si>
+    <t>TC_010</t>
+  </si>
+  <si>
+    <t>Validation message should appear for Uestion label</t>
+  </si>
+  <si>
+    <t>TC_011</t>
+  </si>
+  <si>
+    <t>Validation should appear if minimum limit &gt; 0</t>
+  </si>
+  <si>
+    <t>TC_012</t>
+  </si>
+  <si>
+    <t>Expiry Date should be greater than Start Date</t>
+  </si>
+  <si>
+    <t>TC_013</t>
+  </si>
+  <si>
+    <t>31-11-2026</t>
+  </si>
+  <si>
+    <t>Strat date should be current date or future date</t>
+  </si>
+  <si>
+    <t>TC_014</t>
+  </si>
+  <si>
+    <t>Form should be created if dates are optional</t>
+  </si>
+  <si>
+    <t>TC_015</t>
+  </si>
+  <si>
+    <t>TC_016</t>
+  </si>
+  <si>
+    <t>Question Label validation should appear</t>
+  </si>
+  <si>
+    <t>TC_017</t>
+  </si>
+  <si>
+    <t>Field Type validation should appear</t>
+  </si>
+  <si>
+    <t>TC_018</t>
+  </si>
+  <si>
+    <t>TC_019</t>
+  </si>
+  <si>
+    <t>SQL Injection Test</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>' OR 1=1 --</t>
+  </si>
+  <si>
+    <t>Application should handle malicious input safely</t>
+  </si>
+  <si>
+    <t>TC_020</t>
+  </si>
+  <si>
+    <t>XSS Test</t>
+  </si>
+  <si>
+    <t>alert('XSS')</t>
+  </si>
+  <si>
+    <t>XSS input should be sanitized</t>
+  </si>
+  <si>
+    <t>TC_021</t>
+  </si>
+  <si>
+    <t>Normal Description</t>
+  </si>
+  <si>
+    <t>Complete Details</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>Boundary value should be handled successfully</t>
   </si>
 </sst>
 </file>
@@ -840,7 +1090,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -877,6 +1127,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2607,4 +2858,1025 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC8D3CA3-754F-4C80-BFFE-C010FAB85391}">
+  <dimension ref="A1:O22"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="7" max="7" width="13.453125" customWidth="1"/>
+    <col min="8" max="8" width="11.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" t="s">
+        <v>214</v>
+      </c>
+      <c r="F1" t="s">
+        <v>215</v>
+      </c>
+      <c r="G1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I1" t="s">
+        <v>216</v>
+      </c>
+      <c r="J1" t="s">
+        <v>217</v>
+      </c>
+      <c r="K1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L1" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" t="s">
+        <v>58</v>
+      </c>
+      <c r="N1" t="s">
+        <v>6</v>
+      </c>
+      <c r="O1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D2" t="s">
+        <v>220</v>
+      </c>
+      <c r="E2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2">
+        <v>100</v>
+      </c>
+      <c r="G2" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H2" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I2" t="s">
+        <v>221</v>
+      </c>
+      <c r="J2" t="s">
+        <v>222</v>
+      </c>
+      <c r="K2" t="s">
+        <v>223</v>
+      </c>
+      <c r="L2" t="s">
+        <v>88</v>
+      </c>
+      <c r="M2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" t="s">
+        <v>224</v>
+      </c>
+      <c r="O2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>225</v>
+      </c>
+      <c r="B3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C3" t="s">
+        <v>227</v>
+      </c>
+      <c r="D3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3">
+        <v>500</v>
+      </c>
+      <c r="G3" s="14">
+        <v>46310</v>
+      </c>
+      <c r="H3" s="14">
+        <v>46341</v>
+      </c>
+      <c r="I3" t="s">
+        <v>228</v>
+      </c>
+      <c r="J3" t="s">
+        <v>229</v>
+      </c>
+      <c r="K3" t="s">
+        <v>230</v>
+      </c>
+      <c r="L3" t="s">
+        <v>231</v>
+      </c>
+      <c r="M3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N3" t="s">
+        <v>224</v>
+      </c>
+      <c r="O3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B4" t="s">
+        <v>233</v>
+      </c>
+      <c r="D4" t="s">
+        <v>234</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4">
+        <v>50</v>
+      </c>
+      <c r="G4" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H4" s="14">
+        <v>46315</v>
+      </c>
+      <c r="I4" t="s">
+        <v>235</v>
+      </c>
+      <c r="J4" t="s">
+        <v>236</v>
+      </c>
+      <c r="K4" t="s">
+        <v>237</v>
+      </c>
+      <c r="L4" t="s">
+        <v>238</v>
+      </c>
+      <c r="M4" t="s">
+        <v>35</v>
+      </c>
+      <c r="N4" t="s">
+        <v>224</v>
+      </c>
+      <c r="O4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>239</v>
+      </c>
+      <c r="B5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D5" t="s">
+        <v>220</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5">
+        <v>500</v>
+      </c>
+      <c r="G5" s="14">
+        <v>46310</v>
+      </c>
+      <c r="H5" s="14">
+        <v>46341</v>
+      </c>
+      <c r="I5" t="s">
+        <v>228</v>
+      </c>
+      <c r="K5" t="s">
+        <v>230</v>
+      </c>
+      <c r="L5" t="s">
+        <v>231</v>
+      </c>
+      <c r="M5" t="s">
+        <v>35</v>
+      </c>
+      <c r="N5" t="s">
+        <v>224</v>
+      </c>
+      <c r="O5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>240</v>
+      </c>
+      <c r="C6" t="s">
+        <v>241</v>
+      </c>
+      <c r="D6" t="s">
+        <v>220</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6">
+        <v>100</v>
+      </c>
+      <c r="G6" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H6" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I6" t="s">
+        <v>242</v>
+      </c>
+      <c r="J6" t="s">
+        <v>243</v>
+      </c>
+      <c r="K6" t="s">
+        <v>223</v>
+      </c>
+      <c r="L6" t="s">
+        <v>88</v>
+      </c>
+      <c r="M6" t="s">
+        <v>35</v>
+      </c>
+      <c r="N6" t="s">
+        <v>244</v>
+      </c>
+      <c r="O6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" t="s">
+        <v>246</v>
+      </c>
+      <c r="C7" t="s">
+        <v>247</v>
+      </c>
+      <c r="D7" t="s">
+        <v>220</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7">
+        <v>100</v>
+      </c>
+      <c r="G7" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H7" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I7" t="s">
+        <v>242</v>
+      </c>
+      <c r="J7" t="s">
+        <v>243</v>
+      </c>
+      <c r="K7" t="s">
+        <v>223</v>
+      </c>
+      <c r="L7" t="s">
+        <v>88</v>
+      </c>
+      <c r="M7" t="s">
+        <v>35</v>
+      </c>
+      <c r="N7" t="s">
+        <v>248</v>
+      </c>
+      <c r="O7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C8" t="s">
+        <v>251</v>
+      </c>
+      <c r="D8" t="s">
+        <v>220</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8">
+        <v>100</v>
+      </c>
+      <c r="G8" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H8" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I8" t="s">
+        <v>242</v>
+      </c>
+      <c r="J8" t="s">
+        <v>243</v>
+      </c>
+      <c r="K8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L8" t="s">
+        <v>88</v>
+      </c>
+      <c r="M8" t="s">
+        <v>35</v>
+      </c>
+      <c r="N8" t="s">
+        <v>252</v>
+      </c>
+      <c r="O8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>253</v>
+      </c>
+      <c r="B9" t="s">
+        <v>254</v>
+      </c>
+      <c r="C9" t="s">
+        <v>255</v>
+      </c>
+      <c r="D9" t="s">
+        <v>220</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9">
+        <v>100</v>
+      </c>
+      <c r="G9" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H9" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I9" t="s">
+        <v>242</v>
+      </c>
+      <c r="J9" t="s">
+        <v>243</v>
+      </c>
+      <c r="K9" t="s">
+        <v>223</v>
+      </c>
+      <c r="L9" t="s">
+        <v>88</v>
+      </c>
+      <c r="M9" t="s">
+        <v>35</v>
+      </c>
+      <c r="N9" t="s">
+        <v>256</v>
+      </c>
+      <c r="O9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>257</v>
+      </c>
+      <c r="B10" t="s">
+        <v>258</v>
+      </c>
+      <c r="C10" t="s">
+        <v>259</v>
+      </c>
+      <c r="D10" t="s">
+        <v>220</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10">
+        <v>-10</v>
+      </c>
+      <c r="G10" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H10" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I10" t="s">
+        <v>260</v>
+      </c>
+      <c r="J10" t="s">
+        <v>261</v>
+      </c>
+      <c r="K10" t="s">
+        <v>262</v>
+      </c>
+      <c r="L10" t="s">
+        <v>238</v>
+      </c>
+      <c r="M10" t="s">
+        <v>35</v>
+      </c>
+      <c r="N10" t="s">
+        <v>263</v>
+      </c>
+      <c r="O10" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B11" t="s">
+        <v>258</v>
+      </c>
+      <c r="C11" t="s">
+        <v>259</v>
+      </c>
+      <c r="D11" t="s">
+        <v>220</v>
+      </c>
+      <c r="E11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11">
+        <v>75</v>
+      </c>
+      <c r="G11" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H11" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I11" t="s">
+        <v>260</v>
+      </c>
+      <c r="J11" t="s">
+        <v>261</v>
+      </c>
+      <c r="L11" t="s">
+        <v>238</v>
+      </c>
+      <c r="M11" t="s">
+        <v>35</v>
+      </c>
+      <c r="N11" t="s">
+        <v>265</v>
+      </c>
+      <c r="O11" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>266</v>
+      </c>
+      <c r="B12" t="s">
+        <v>258</v>
+      </c>
+      <c r="C12" t="s">
+        <v>259</v>
+      </c>
+      <c r="D12" t="s">
+        <v>220</v>
+      </c>
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H12" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I12" t="s">
+        <v>260</v>
+      </c>
+      <c r="J12" t="s">
+        <v>261</v>
+      </c>
+      <c r="K12" t="s">
+        <v>262</v>
+      </c>
+      <c r="L12" t="s">
+        <v>238</v>
+      </c>
+      <c r="M12" t="s">
+        <v>35</v>
+      </c>
+      <c r="N12" t="s">
+        <v>267</v>
+      </c>
+      <c r="O12" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>268</v>
+      </c>
+      <c r="B13" t="s">
+        <v>258</v>
+      </c>
+      <c r="C13" t="s">
+        <v>259</v>
+      </c>
+      <c r="D13" t="s">
+        <v>220</v>
+      </c>
+      <c r="E13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13">
+        <v>100</v>
+      </c>
+      <c r="G13" s="14">
+        <v>46326</v>
+      </c>
+      <c r="H13" s="14">
+        <v>46305</v>
+      </c>
+      <c r="I13" t="s">
+        <v>260</v>
+      </c>
+      <c r="J13" t="s">
+        <v>261</v>
+      </c>
+      <c r="K13" t="s">
+        <v>262</v>
+      </c>
+      <c r="L13" t="s">
+        <v>238</v>
+      </c>
+      <c r="M13" t="s">
+        <v>35</v>
+      </c>
+      <c r="N13" t="s">
+        <v>269</v>
+      </c>
+      <c r="O13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>270</v>
+      </c>
+      <c r="B14" t="s">
+        <v>258</v>
+      </c>
+      <c r="C14" t="s">
+        <v>259</v>
+      </c>
+      <c r="D14" t="s">
+        <v>220</v>
+      </c>
+      <c r="E14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14">
+        <v>100</v>
+      </c>
+      <c r="G14" s="14">
+        <v>9436</v>
+      </c>
+      <c r="H14" t="s">
+        <v>271</v>
+      </c>
+      <c r="I14" t="s">
+        <v>260</v>
+      </c>
+      <c r="J14" t="s">
+        <v>261</v>
+      </c>
+      <c r="K14" t="s">
+        <v>262</v>
+      </c>
+      <c r="L14" t="s">
+        <v>238</v>
+      </c>
+      <c r="M14" t="s">
+        <v>35</v>
+      </c>
+      <c r="N14" t="s">
+        <v>272</v>
+      </c>
+      <c r="O14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>273</v>
+      </c>
+      <c r="B15" t="s">
+        <v>258</v>
+      </c>
+      <c r="C15" t="s">
+        <v>259</v>
+      </c>
+      <c r="D15" t="s">
+        <v>220</v>
+      </c>
+      <c r="E15" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15">
+        <v>100</v>
+      </c>
+      <c r="I15" t="s">
+        <v>260</v>
+      </c>
+      <c r="J15" t="s">
+        <v>261</v>
+      </c>
+      <c r="K15" t="s">
+        <v>262</v>
+      </c>
+      <c r="L15" t="s">
+        <v>238</v>
+      </c>
+      <c r="M15" t="s">
+        <v>35</v>
+      </c>
+      <c r="N15" t="s">
+        <v>274</v>
+      </c>
+      <c r="O15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>275</v>
+      </c>
+      <c r="B16" t="s">
+        <v>258</v>
+      </c>
+      <c r="C16" t="s">
+        <v>259</v>
+      </c>
+      <c r="D16" t="s">
+        <v>220</v>
+      </c>
+      <c r="E16" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16">
+        <v>100</v>
+      </c>
+      <c r="G16" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H16" s="14">
+        <v>46326</v>
+      </c>
+      <c r="J16" t="s">
+        <v>243</v>
+      </c>
+      <c r="K16" t="s">
+        <v>223</v>
+      </c>
+      <c r="L16" t="s">
+        <v>88</v>
+      </c>
+      <c r="M16" t="s">
+        <v>35</v>
+      </c>
+      <c r="N16" t="s">
+        <v>224</v>
+      </c>
+      <c r="O16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>276</v>
+      </c>
+      <c r="B17" t="s">
+        <v>258</v>
+      </c>
+      <c r="C17" t="s">
+        <v>259</v>
+      </c>
+      <c r="D17" t="s">
+        <v>220</v>
+      </c>
+      <c r="E17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17">
+        <v>100</v>
+      </c>
+      <c r="G17" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H17" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I17" t="s">
+        <v>221</v>
+      </c>
+      <c r="J17" t="s">
+        <v>243</v>
+      </c>
+      <c r="L17" t="s">
+        <v>88</v>
+      </c>
+      <c r="M17" t="s">
+        <v>35</v>
+      </c>
+      <c r="N17" t="s">
+        <v>277</v>
+      </c>
+      <c r="O17" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>278</v>
+      </c>
+      <c r="B18" t="s">
+        <v>258</v>
+      </c>
+      <c r="C18" t="s">
+        <v>259</v>
+      </c>
+      <c r="D18" t="s">
+        <v>220</v>
+      </c>
+      <c r="E18" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18">
+        <v>100</v>
+      </c>
+      <c r="G18" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H18" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I18" t="s">
+        <v>221</v>
+      </c>
+      <c r="J18" t="s">
+        <v>243</v>
+      </c>
+      <c r="K18" t="s">
+        <v>223</v>
+      </c>
+      <c r="M18" t="s">
+        <v>35</v>
+      </c>
+      <c r="N18" t="s">
+        <v>279</v>
+      </c>
+      <c r="O18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>280</v>
+      </c>
+      <c r="B19" t="s">
+        <v>258</v>
+      </c>
+      <c r="C19" t="s">
+        <v>259</v>
+      </c>
+      <c r="D19" t="s">
+        <v>220</v>
+      </c>
+      <c r="E19" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19">
+        <v>100</v>
+      </c>
+      <c r="G19" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H19" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I19" t="s">
+        <v>221</v>
+      </c>
+      <c r="J19" t="s">
+        <v>243</v>
+      </c>
+      <c r="K19" t="s">
+        <v>223</v>
+      </c>
+      <c r="L19" t="s">
+        <v>88</v>
+      </c>
+      <c r="M19" t="s">
+        <v>21</v>
+      </c>
+      <c r="N19" t="s">
+        <v>224</v>
+      </c>
+      <c r="O19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>281</v>
+      </c>
+      <c r="B20" t="s">
+        <v>258</v>
+      </c>
+      <c r="C20" t="s">
+        <v>282</v>
+      </c>
+      <c r="D20" t="s">
+        <v>220</v>
+      </c>
+      <c r="E20" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20">
+        <v>100</v>
+      </c>
+      <c r="G20" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H20" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I20" t="s">
+        <v>221</v>
+      </c>
+      <c r="J20" t="s">
+        <v>283</v>
+      </c>
+      <c r="K20" t="s">
+        <v>284</v>
+      </c>
+      <c r="L20" t="s">
+        <v>88</v>
+      </c>
+      <c r="M20" t="s">
+        <v>35</v>
+      </c>
+      <c r="N20" t="s">
+        <v>285</v>
+      </c>
+      <c r="O20" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>286</v>
+      </c>
+      <c r="B21" t="s">
+        <v>258</v>
+      </c>
+      <c r="C21" t="s">
+        <v>287</v>
+      </c>
+      <c r="D21" t="s">
+        <v>220</v>
+      </c>
+      <c r="E21" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21">
+        <v>100</v>
+      </c>
+      <c r="G21" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H21" s="14">
+        <v>46326</v>
+      </c>
+      <c r="I21" t="s">
+        <v>221</v>
+      </c>
+      <c r="J21" t="s">
+        <v>283</v>
+      </c>
+      <c r="K21" t="s">
+        <v>288</v>
+      </c>
+      <c r="L21" t="s">
+        <v>88</v>
+      </c>
+      <c r="M21" t="s">
+        <v>35</v>
+      </c>
+      <c r="N21" t="s">
+        <v>289</v>
+      </c>
+      <c r="O21" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>290</v>
+      </c>
+      <c r="B22" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" t="s">
+        <v>291</v>
+      </c>
+      <c r="D22" t="s">
+        <v>220</v>
+      </c>
+      <c r="E22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22">
+        <v>999999</v>
+      </c>
+      <c r="G22" s="14">
+        <v>46305</v>
+      </c>
+      <c r="H22" s="14">
+        <v>46387</v>
+      </c>
+      <c r="I22" t="s">
+        <v>221</v>
+      </c>
+      <c r="J22" t="s">
+        <v>292</v>
+      </c>
+      <c r="K22" t="s">
+        <v>293</v>
+      </c>
+      <c r="L22" t="s">
+        <v>238</v>
+      </c>
+      <c r="M22" t="s">
+        <v>35</v>
+      </c>
+      <c r="N22" t="s">
+        <v>294</v>
+      </c>
+      <c r="O22" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>